<commit_message>
refactor: alinhar vocabulario de dominio (Aluno), estrita validacao de colunas e robustez CSV
</commit_message>
<xml_diff>
--- a/modelo_alunos.xlsx
+++ b/modelo_alunos.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,10 +29,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -62,15 +58,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -438,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -457,42 +447,6 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Maria da Silva</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>529.982.247-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>João dos Santos</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>111.444.777-35</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Ana Paula do Nascimento</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>012.345.678-90</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>